<commit_message>
Id to HFD AIC calculated
</commit_message>
<xml_diff>
--- a/output/female_HFD_average_of_ECG_per_age_range_kmax_10000and16000and25000_cycle_step_50_num_k_50.xlsx
+++ b/output/female_HFD_average_of_ECG_per_age_range_kmax_10000and16000and25000_cycle_step_50_num_k_50.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ECGBiologicalAge\HeartAge\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{1CABE355-718D-4A46-9872-8B0EF6A08192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85F6F4A7-0C69-4742-9603-6E8B0F8BEA81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="15000" xr2:uid="{EEA73793-FFC9-4D0F-B3C6-A2F879ADB122}"/>
   </bookViews>
@@ -680,7 +680,7 @@
                   </a:sysClr>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Higuchi fractal dimension (HFD) per each age range for all males</a:t>
+              <a:t>Higuchi fractal dimension (HFD) per each age range for all females </a:t>
             </a:r>
             <a:endParaRPr lang="uk-UA" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -760,49 +760,49 @@
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
+                  <c:v>18 - 19</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>20 - 24</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
+                  <c:v>25 - 29</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30 - 34</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>35 - 39</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40 - 44</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>45 - 49</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>30 - 34</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>25 - 29</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>18 - 19</c:v>
-                </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
+                  <c:v>50 - 54</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>55 - 59</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>60 - 64</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>50 - 54</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>40 - 44</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>35 - 39</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>55 - 59</c:v>
-                </c:pt>
                 <c:pt idx="10">
+                  <c:v>65 - 69</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>70 - 74</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>75 - 79</c:v>
                 </c:pt>
-                <c:pt idx="11">
-                  <c:v>65 - 69</c:v>
-                </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="13">
+                  <c:v>80 - 84</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>85 - 92</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>70 - 74</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>80 - 84</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -814,49 +814,49 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
+                  <c:v>1.788</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1.786</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
+                  <c:v>1.786</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.7849999999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>1.7809999999999999</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.7849999999999999</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
+                  <c:v>1.7809999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.7809999999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.784</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.778</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.766</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.782</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.778</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.7949999999999999</c:v>
+                </c:pt>
+                <c:pt idx="13">
                   <c:v>1.786</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.788</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.766</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.784</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.7809999999999999</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.7809999999999999</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.778</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.7949999999999999</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.782</c:v>
-                </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="14">
                   <c:v>1.7869999999999999</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.778</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1.786</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -900,49 +900,49 @@
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
+                  <c:v>18 - 19</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>20 - 24</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
+                  <c:v>25 - 29</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30 - 34</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>35 - 39</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40 - 44</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>45 - 49</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>30 - 34</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>25 - 29</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>18 - 19</c:v>
-                </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
+                  <c:v>50 - 54</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>55 - 59</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>60 - 64</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>50 - 54</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>40 - 44</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>35 - 39</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>55 - 59</c:v>
-                </c:pt>
                 <c:pt idx="10">
+                  <c:v>65 - 69</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>70 - 74</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>75 - 79</c:v>
                 </c:pt>
-                <c:pt idx="11">
-                  <c:v>65 - 69</c:v>
-                </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="13">
+                  <c:v>80 - 84</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>85 - 92</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>70 - 74</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>80 - 84</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -954,46 +954,46 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
+                  <c:v>1.8169999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1.8149999999999999</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
+                  <c:v>1.8149999999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.8140000000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>1.8109999999999999</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.8140000000000001</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
+                  <c:v>1.8109999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.8109999999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.8129999999999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.81</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.7989999999999999</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.8120000000000001</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.8069999999999999</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.8220000000000001</c:v>
+                </c:pt>
+                <c:pt idx="13">
                   <c:v>1.8149999999999999</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.8169999999999999</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.7989999999999999</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.8129999999999999</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.8109999999999999</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.8109999999999999</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.81</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.8220000000000001</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.8120000000000001</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.8149999999999999</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>1.8069999999999999</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>1.8149999999999999</c:v>
@@ -1040,49 +1040,49 @@
               <c:strCache>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
+                  <c:v>18 - 19</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>20 - 24</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
+                  <c:v>25 - 29</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30 - 34</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>35 - 39</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>40 - 44</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>45 - 49</c:v>
                 </c:pt>
-                <c:pt idx="2">
-                  <c:v>30 - 34</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>25 - 29</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>18 - 19</c:v>
-                </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="7">
+                  <c:v>50 - 54</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>55 - 59</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>60 - 64</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>50 - 54</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>40 - 44</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>35 - 39</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>55 - 59</c:v>
-                </c:pt>
                 <c:pt idx="10">
+                  <c:v>65 - 69</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>70 - 74</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>75 - 79</c:v>
                 </c:pt>
-                <c:pt idx="11">
-                  <c:v>65 - 69</c:v>
-                </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="13">
+                  <c:v>80 - 84</c:v>
+                </c:pt>
+                <c:pt idx="14">
                   <c:v>85 - 92</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>70 - 74</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>80 - 84</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1094,49 +1094,49 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
+                  <c:v>1.8109999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1.8169999999999999</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
+                  <c:v>1.8140000000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>1.8149999999999999</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="4">
+                  <c:v>1.81</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.8129999999999999</c:v>
+                </c:pt>
+                <c:pt idx="6">
                   <c:v>1.8149999999999999</c:v>
                 </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.8140000000000001</c:v>
-                </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="7">
                   <c:v>1.8109999999999999</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="8">
+                  <c:v>1.7989999999999999</c:v>
+                </c:pt>
+                <c:pt idx="9">
                   <c:v>1.8109999999999999</c:v>
                 </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.8109999999999999</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.8129999999999999</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.81</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.7989999999999999</c:v>
-                </c:pt>
                 <c:pt idx="10">
+                  <c:v>1.8069999999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.8149999999999999</c:v>
+                </c:pt>
+                <c:pt idx="12">
                   <c:v>1.8120000000000001</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>1.8069999999999999</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.8220000000000001</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>1.8149999999999999</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.8149999999999999</c:v>
+                  <c:v>1.8220000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2448,195 +2448,195 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B2">
-        <v>1.786</v>
+        <v>1.788</v>
       </c>
       <c r="C2">
-        <v>1.8149999999999999</v>
+        <v>1.8169999999999999</v>
       </c>
       <c r="D2">
-        <v>1.8169999999999999</v>
+        <v>1.8109999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B3">
-        <v>1.7809999999999999</v>
+        <v>1.786</v>
       </c>
       <c r="C3">
-        <v>1.8109999999999999</v>
+        <v>1.8149999999999999</v>
       </c>
       <c r="D3">
-        <v>1.8149999999999999</v>
+        <v>1.8169999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4">
-        <v>1.7849999999999999</v>
+        <v>1.786</v>
       </c>
       <c r="C4">
+        <v>1.8149999999999999</v>
+      </c>
+      <c r="D4">
         <v>1.8140000000000001</v>
-      </c>
-      <c r="D4">
-        <v>1.8149999999999999</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5">
-        <v>1.786</v>
+        <v>1.7849999999999999</v>
       </c>
       <c r="C5">
+        <v>1.8140000000000001</v>
+      </c>
+      <c r="D5">
         <v>1.8149999999999999</v>
-      </c>
-      <c r="D5">
-        <v>1.8140000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B6">
-        <v>1.788</v>
+        <v>1.7809999999999999</v>
       </c>
       <c r="C6">
-        <v>1.8169999999999999</v>
+        <v>1.8109999999999999</v>
       </c>
       <c r="D6">
-        <v>1.8109999999999999</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B7">
-        <v>1.766</v>
+        <v>1.7809999999999999</v>
       </c>
       <c r="C7">
-        <v>1.7989999999999999</v>
+        <v>1.8109999999999999</v>
       </c>
       <c r="D7">
-        <v>1.8109999999999999</v>
+        <v>1.8129999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B8">
-        <v>1.784</v>
+        <v>1.7809999999999999</v>
       </c>
       <c r="C8">
-        <v>1.8129999999999999</v>
+        <v>1.8109999999999999</v>
       </c>
       <c r="D8">
-        <v>1.8109999999999999</v>
+        <v>1.8149999999999999</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9">
-        <v>1.7809999999999999</v>
+        <v>1.784</v>
       </c>
       <c r="C9">
+        <v>1.8129999999999999</v>
+      </c>
+      <c r="D9">
         <v>1.8109999999999999</v>
-      </c>
-      <c r="D9">
-        <v>1.8129999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10">
-        <v>1.7809999999999999</v>
+        <v>1.778</v>
       </c>
       <c r="C10">
-        <v>1.8109999999999999</v>
+        <v>1.81</v>
       </c>
       <c r="D10">
-        <v>1.81</v>
+        <v>1.7989999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B11">
-        <v>1.778</v>
+        <v>1.766</v>
       </c>
       <c r="C11">
-        <v>1.81</v>
+        <v>1.7989999999999999</v>
       </c>
       <c r="D11">
-        <v>1.7989999999999999</v>
+        <v>1.8109999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12">
-        <v>1.7949999999999999</v>
+        <v>1.782</v>
       </c>
       <c r="C12">
-        <v>1.8220000000000001</v>
+        <v>1.8120000000000001</v>
       </c>
       <c r="D12">
-        <v>1.8120000000000001</v>
+        <v>1.8069999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B13">
-        <v>1.782</v>
+        <v>1.778</v>
       </c>
       <c r="C13">
-        <v>1.8120000000000001</v>
+        <v>1.8069999999999999</v>
       </c>
       <c r="D13">
-        <v>1.8069999999999999</v>
+        <v>1.8149999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B14">
-        <v>1.7869999999999999</v>
+        <v>1.7949999999999999</v>
       </c>
       <c r="C14">
-        <v>1.8149999999999999</v>
+        <v>1.8220000000000001</v>
       </c>
       <c r="D14">
-        <v>1.8220000000000001</v>
+        <v>1.8120000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15">
-        <v>1.778</v>
+        <v>1.786</v>
       </c>
       <c r="C15">
-        <v>1.8069999999999999</v>
+        <v>1.8149999999999999</v>
       </c>
       <c r="D15">
         <v>1.8149999999999999</v>
@@ -2644,19 +2644,22 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B16">
-        <v>1.786</v>
+        <v>1.7869999999999999</v>
       </c>
       <c r="C16">
         <v>1.8149999999999999</v>
       </c>
       <c r="D16">
-        <v>1.8149999999999999</v>
+        <v>1.8220000000000001</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D16">
+    <sortCondition ref="A2:A16"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>